<commit_message>
feat: add project report and update output files for improved documentation and data handling
</commit_message>
<xml_diff>
--- a/data/output/output.xlsx
+++ b/data/output/output.xlsx
@@ -429,13 +429,13 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="26" customWidth="1" min="6" max="6"/>
     <col width="23" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
@@ -492,7 +492,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ધામણા મોટા</t>
+          <t>Dhanpur</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -502,7 +502,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>5,275.00 ચો.મી.</t>
+          <t>5,275.00 sq.mt.</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -515,9 +515,21 @@
           <t>iORA/31/02/112/25/2026</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>141/2026</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>04047 Square Meters</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>21/01/2026</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -525,7 +537,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ધાનપુર મોટા</t>
+          <t>Rampura Mota</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -535,7 +547,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>34,576.00 sq.mt.</t>
+          <t>34,576.00 ચો.મી.</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -570,17 +582,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>ધામણુ મોટા</t>
+          <t>Rampura Mota</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>256</t>
+          <t>257</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>16,510.00 ચો.મી.</t>
+          <t>16,534.00 sq.mt.</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -590,17 +602,17 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>iORA/31/02/112/8/2026</t>
+          <t>iORA/31/02/112/7/2026</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>854/2025</t>
+          <t>837/2025</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>16959 sq.mt.</t>
+          <t>16792 sq.mt.</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -615,42 +627,30 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>ધાનપુર</t>
+          <t>Rampura Mota</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>257</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>16,534.00 sq.mt.</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>07/01/2026</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>iORA/31/02/112/7/2026</t>
-        </is>
-      </c>
+          <t>256</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
-          <t>837/2025</t>
+          <t>854/2025</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>16792 sq.mt.</t>
+          <t>16959 sq.mt. (4.19 Acre)</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>28/05/2025</t>
+          <t>02/06/2025</t>
         </is>
       </c>
     </row>

</xml_diff>